<commit_message>
Advance filters & Conditional Formatting
</commit_message>
<xml_diff>
--- a/Excel/8. Advance Filters/Advanced+Filters.xlsx
+++ b/Excel/8. Advance Filters/Advanced+Filters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DC_DDS_04\Excel\8. Advance Filters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A628180-D65A-429F-9CDA-DBED05D19F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EDFA2D-D37C-456D-BA97-56E8F950C754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="4" xr2:uid="{29745A60-A6D0-4A7B-AF84-F627A3EF9D41}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="6" xr2:uid="{29745A60-A6D0-4A7B-AF84-F627A3EF9D41}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="5" r:id="rId1"/>
@@ -26,6 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">AND!$A$1:$I$299</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Between!$A$1:$I$299</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$I$299</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">OR!$A$1:$I$299</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Simple Example'!$A$1:$I$299</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Unique!$C:$C</definedName>
@@ -37,6 +38,7 @@
     <definedName name="_xlnm.Criteria" localSheetId="6">Wildcard!#REF!</definedName>
     <definedName name="_xlnm.Extract" localSheetId="3">AND!$K$15:$S$15</definedName>
     <definedName name="_xlnm.Extract" localSheetId="5">Between!#REF!</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="0">AND!$K$16:$S$16</definedName>
     <definedName name="_xlnm.Extract" localSheetId="4">OR!$K$14:$S$14</definedName>
     <definedName name="_xlnm.Extract" localSheetId="1">'Simple Example'!$K$15:$S$15</definedName>
     <definedName name="_xlnm.Extract" localSheetId="8">Unique!#REF!</definedName>
@@ -1998,7 +2000,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2018,6 +2020,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2353,10 +2363,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2381,6 +2392,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2408,14 +2423,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2742,6 +2753,15 @@
     <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -11504,12 +11524,12 @@
       <c r="I2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="26" t="s">
         <v>630</v>
       </c>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="24"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11539,10 +11559,10 @@
       <c r="I3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="27"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="31"/>
     </row>
     <row r="4" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -11572,10 +11592,10 @@
       <c r="I4" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="31"/>
       <c r="O4" s="19"/>
       <c r="P4" s="19"/>
       <c r="Q4" s="19"/>
@@ -11611,10 +11631,10 @@
       <c r="I5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="25"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="31"/>
       <c r="O5" s="19"/>
       <c r="P5" s="19"/>
       <c r="Q5" s="19"/>
@@ -11647,10 +11667,10 @@
       <c r="I6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="25"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="27"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
+      <c r="N6" s="31"/>
       <c r="O6" s="19"/>
       <c r="P6" s="19"/>
       <c r="Q6" s="19"/>
@@ -11683,10 +11703,10 @@
       <c r="I7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="28"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="29"/>
-      <c r="N7" s="30"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="34"/>
       <c r="O7" s="19"/>
       <c r="P7" s="19"/>
       <c r="Q7" s="19"/>
@@ -11786,15 +11806,7 @@
       <c r="K10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L10" s="31"/>
-      <c r="M10" s="32"/>
-      <c r="N10" s="32"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="32"/>
-      <c r="R10" s="32"/>
-      <c r="S10" s="32"/>
-      <c r="T10" s="32"/>
+      <c r="L10" s="17"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -11828,15 +11840,6 @@
         <f>"=Sarah Johnson"</f>
         <v>=Sarah Johnson</v>
       </c>
-      <c r="L11" s="32"/>
-      <c r="M11" s="32"/>
-      <c r="N11" s="32"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="32"/>
-      <c r="Q11" s="32"/>
-      <c r="R11" s="32"/>
-      <c r="S11" s="32"/>
-      <c r="T11" s="32"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
@@ -11866,15 +11869,6 @@
       <c r="I12" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="L12" s="32"/>
-      <c r="M12" s="32"/>
-      <c r="N12" s="32"/>
-      <c r="O12" s="32"/>
-      <c r="P12" s="32"/>
-      <c r="Q12" s="32"/>
-      <c r="R12" s="32"/>
-      <c r="S12" s="32"/>
-      <c r="T12" s="32"/>
     </row>
     <row r="13" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
@@ -11904,15 +11898,15 @@
       <c r="I13" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="31"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="31"/>
-      <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="31"/>
-      <c r="T13" s="31"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17"/>
+      <c r="T13" s="17"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -11942,15 +11936,8 @@
       <c r="I14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L14" s="32"/>
-      <c r="M14" s="32"/>
-      <c r="N14" s="32"/>
-      <c r="O14" s="34"/>
-      <c r="P14" s="34"/>
-      <c r="Q14" s="32"/>
-      <c r="R14" s="32"/>
-      <c r="S14" s="32"/>
-      <c r="T14" s="32"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="23"/>
     </row>
     <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
@@ -11980,36 +11967,16 @@
       <c r="I15" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="P15" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="S15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="T15" s="32"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17"/>
+    </row>
+    <row r="16" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>55</v>
       </c>
@@ -12037,34 +12004,33 @@
       <c r="I16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="N16" s="11">
-        <v>43184</v>
-      </c>
-      <c r="O16" s="11">
-        <v>43188</v>
-      </c>
-      <c r="P16" s="10">
-        <v>24716</v>
-      </c>
-      <c r="Q16" s="10">
+      <c r="L16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R16" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="S16" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="T16" s="32"/>
+      <c r="Q16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T16" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
@@ -12094,34 +12060,33 @@
       <c r="I17" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="L17" s="10" t="s">
-        <v>101</v>
+      <c r="L17" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="M17" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="N17" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N17" s="11">
-        <v>45061</v>
-      </c>
       <c r="O17" s="11">
-        <v>45068</v>
-      </c>
-      <c r="P17" s="10">
-        <v>57920</v>
+        <v>43184</v>
+      </c>
+      <c r="P17" s="11">
+        <v>43188</v>
       </c>
       <c r="Q17" s="10">
-        <v>1</v>
-      </c>
-      <c r="R17" s="10" t="s">
-        <v>18</v>
+        <v>24716</v>
+      </c>
+      <c r="R17" s="10">
+        <v>4</v>
       </c>
       <c r="S17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="T17" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="T17" s="32"/>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -12151,34 +12116,33 @@
       <c r="I18" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="L18" s="10" t="s">
-        <v>128</v>
+      <c r="L18" s="9" t="s">
+        <v>100</v>
       </c>
       <c r="M18" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="N18" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N18" s="11">
-        <v>44044</v>
-      </c>
       <c r="O18" s="11">
-        <v>44049</v>
-      </c>
-      <c r="P18" s="10">
-        <v>66354</v>
+        <v>45061</v>
+      </c>
+      <c r="P18" s="11">
+        <v>45068</v>
       </c>
       <c r="Q18" s="10">
+        <v>57920</v>
+      </c>
+      <c r="R18" s="10">
         <v>1</v>
       </c>
-      <c r="R18" s="10" t="s">
-        <v>61</v>
-      </c>
       <c r="S18" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="T18" s="32"/>
+        <v>18</v>
+      </c>
+      <c r="T18" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -12208,34 +12172,33 @@
       <c r="I19" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K19" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="L19" s="10" t="s">
-        <v>130</v>
+      <c r="L19" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="M19" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N19" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N19" s="11">
-        <v>43362</v>
-      </c>
       <c r="O19" s="11">
-        <v>43369</v>
-      </c>
-      <c r="P19" s="10">
-        <v>11908</v>
+        <v>44044</v>
+      </c>
+      <c r="P19" s="11">
+        <v>44049</v>
       </c>
       <c r="Q19" s="10">
-        <v>3</v>
-      </c>
-      <c r="R19" s="10" t="s">
-        <v>13</v>
+        <v>66354</v>
+      </c>
+      <c r="R19" s="10">
+        <v>1</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="T19" s="32"/>
+        <v>61</v>
+      </c>
+      <c r="T19" s="12" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
@@ -12265,34 +12228,33 @@
       <c r="I20" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="L20" s="10" t="s">
-        <v>132</v>
+      <c r="L20" s="9" t="s">
+        <v>129</v>
       </c>
       <c r="M20" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="N20" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N20" s="11">
-        <v>45021</v>
-      </c>
       <c r="O20" s="11">
-        <v>45026</v>
-      </c>
-      <c r="P20" s="10">
-        <v>33491</v>
+        <v>43362</v>
+      </c>
+      <c r="P20" s="11">
+        <v>43369</v>
       </c>
       <c r="Q20" s="10">
-        <v>2</v>
-      </c>
-      <c r="R20" s="10" t="s">
-        <v>38</v>
+        <v>11908</v>
+      </c>
+      <c r="R20" s="10">
+        <v>3</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="T20" s="32"/>
+        <v>13</v>
+      </c>
+      <c r="T20" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -12322,34 +12284,33 @@
       <c r="I21" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K21" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="L21" s="10" t="s">
-        <v>199</v>
+      <c r="L21" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="M21" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="N21" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N21" s="11">
-        <v>44093</v>
-      </c>
       <c r="O21" s="11">
-        <v>44096</v>
-      </c>
-      <c r="P21" s="10">
-        <v>35171</v>
+        <v>45021</v>
+      </c>
+      <c r="P21" s="11">
+        <v>45026</v>
       </c>
       <c r="Q21" s="10">
-        <v>3</v>
-      </c>
-      <c r="R21" s="10" t="s">
+        <v>33491</v>
+      </c>
+      <c r="R21" s="10">
+        <v>2</v>
+      </c>
+      <c r="S21" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="S21" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="T21" s="32"/>
+      <c r="T21" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
@@ -12379,34 +12340,33 @@
       <c r="I22" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K22" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="L22" s="10" t="s">
-        <v>217</v>
+      <c r="L22" s="9" t="s">
+        <v>198</v>
       </c>
       <c r="M22" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="N22" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N22" s="11">
-        <v>43626</v>
-      </c>
       <c r="O22" s="11">
-        <v>43628</v>
-      </c>
-      <c r="P22" s="10">
-        <v>15391</v>
+        <v>44093</v>
+      </c>
+      <c r="P22" s="11">
+        <v>44096</v>
       </c>
       <c r="Q22" s="10">
-        <v>5</v>
-      </c>
-      <c r="R22" s="10" t="s">
-        <v>57</v>
+        <v>35171</v>
+      </c>
+      <c r="R22" s="10">
+        <v>3</v>
       </c>
       <c r="S22" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="T22" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T22" s="32"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -12436,34 +12396,33 @@
       <c r="I23" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K23" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="L23" s="10" t="s">
-        <v>249</v>
+      <c r="L23" s="9" t="s">
+        <v>216</v>
       </c>
       <c r="M23" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="N23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N23" s="11">
-        <v>43732</v>
-      </c>
       <c r="O23" s="11">
-        <v>43738</v>
-      </c>
-      <c r="P23" s="10">
-        <v>58310</v>
+        <v>43626</v>
+      </c>
+      <c r="P23" s="11">
+        <v>43628</v>
       </c>
       <c r="Q23" s="10">
+        <v>15391</v>
+      </c>
+      <c r="R23" s="10">
         <v>5</v>
       </c>
-      <c r="R23" s="10" t="s">
-        <v>13</v>
-      </c>
       <c r="S23" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="T23" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T23" s="32"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
@@ -12493,34 +12452,33 @@
       <c r="I24" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K24" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="L24" s="10" t="s">
-        <v>279</v>
+      <c r="L24" s="9" t="s">
+        <v>248</v>
       </c>
       <c r="M24" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="N24" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N24" s="11">
-        <v>44885</v>
-      </c>
       <c r="O24" s="11">
-        <v>44889</v>
-      </c>
-      <c r="P24" s="10">
-        <v>60800</v>
+        <v>43732</v>
+      </c>
+      <c r="P24" s="11">
+        <v>43738</v>
       </c>
       <c r="Q24" s="10">
-        <v>3</v>
-      </c>
-      <c r="R24" s="10" t="s">
-        <v>18</v>
+        <v>58310</v>
+      </c>
+      <c r="R24" s="10">
+        <v>5</v>
       </c>
       <c r="S24" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="T24" s="32"/>
+        <v>13</v>
+      </c>
+      <c r="T24" s="12" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -12550,34 +12508,33 @@
       <c r="I25" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K25" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="L25" s="10" t="s">
-        <v>291</v>
+      <c r="L25" s="9" t="s">
+        <v>278</v>
       </c>
       <c r="M25" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="N25" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N25" s="11">
-        <v>44482</v>
-      </c>
       <c r="O25" s="11">
-        <v>44483</v>
-      </c>
-      <c r="P25" s="10">
-        <v>24405</v>
+        <v>44885</v>
+      </c>
+      <c r="P25" s="11">
+        <v>44889</v>
       </c>
       <c r="Q25" s="10">
-        <v>5</v>
-      </c>
-      <c r="R25" s="10" t="s">
-        <v>38</v>
+        <v>60800</v>
+      </c>
+      <c r="R25" s="10">
+        <v>3</v>
       </c>
       <c r="S25" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="T25" s="32"/>
+        <v>18</v>
+      </c>
+      <c r="T25" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -12607,34 +12564,33 @@
       <c r="I26" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K26" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="L26" s="10" t="s">
-        <v>315</v>
+      <c r="L26" s="9" t="s">
+        <v>290</v>
       </c>
       <c r="M26" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="N26" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N26" s="11">
-        <v>44085</v>
-      </c>
       <c r="O26" s="11">
-        <v>44089</v>
-      </c>
-      <c r="P26" s="10">
-        <v>50955</v>
+        <v>44482</v>
+      </c>
+      <c r="P26" s="11">
+        <v>44483</v>
       </c>
       <c r="Q26" s="10">
-        <v>1</v>
-      </c>
-      <c r="R26" s="10" t="s">
+        <v>24405</v>
+      </c>
+      <c r="R26" s="10">
+        <v>5</v>
+      </c>
+      <c r="S26" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="S26" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="T26" s="32"/>
+      <c r="T26" s="12" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -12664,34 +12620,33 @@
       <c r="I27" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K27" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="L27" s="10" t="s">
-        <v>349</v>
+      <c r="L27" s="9" t="s">
+        <v>314</v>
       </c>
       <c r="M27" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="N27" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N27" s="11">
-        <v>43822</v>
-      </c>
       <c r="O27" s="11">
-        <v>43826</v>
-      </c>
-      <c r="P27" s="10">
-        <v>36641</v>
+        <v>44085</v>
+      </c>
+      <c r="P27" s="11">
+        <v>44089</v>
       </c>
       <c r="Q27" s="10">
-        <v>3</v>
-      </c>
-      <c r="R27" s="10" t="s">
-        <v>13</v>
+        <v>50955</v>
+      </c>
+      <c r="R27" s="10">
+        <v>1</v>
       </c>
       <c r="S27" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="T27" s="32"/>
+        <v>38</v>
+      </c>
+      <c r="T27" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -12721,34 +12676,33 @@
       <c r="I28" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="K28" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="L28" s="10" t="s">
-        <v>459</v>
+      <c r="L28" s="9" t="s">
+        <v>348</v>
       </c>
       <c r="M28" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="N28" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N28" s="11">
-        <v>43979</v>
-      </c>
       <c r="O28" s="11">
-        <v>43982</v>
-      </c>
-      <c r="P28" s="10">
-        <v>73403</v>
+        <v>43822</v>
+      </c>
+      <c r="P28" s="11">
+        <v>43826</v>
       </c>
       <c r="Q28" s="10">
-        <v>5</v>
-      </c>
-      <c r="R28" s="10" t="s">
-        <v>18</v>
+        <v>36641</v>
+      </c>
+      <c r="R28" s="10">
+        <v>3</v>
       </c>
       <c r="S28" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="T28" s="32"/>
+        <v>13</v>
+      </c>
+      <c r="T28" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -12778,34 +12732,33 @@
       <c r="I29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K29" s="9" t="s">
-        <v>544</v>
-      </c>
-      <c r="L29" s="10" t="s">
-        <v>545</v>
+      <c r="L29" s="9" t="s">
+        <v>458</v>
       </c>
       <c r="M29" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="N29" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N29" s="11">
-        <v>44522</v>
-      </c>
       <c r="O29" s="11">
-        <v>44528</v>
-      </c>
-      <c r="P29" s="10">
-        <v>12466</v>
+        <v>43979</v>
+      </c>
+      <c r="P29" s="11">
+        <v>43982</v>
       </c>
       <c r="Q29" s="10">
-        <v>3</v>
-      </c>
-      <c r="R29" s="10" t="s">
-        <v>61</v>
+        <v>73403</v>
+      </c>
+      <c r="R29" s="10">
+        <v>5</v>
       </c>
       <c r="S29" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="T29" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T29" s="32"/>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -12835,34 +12788,33 @@
       <c r="I30" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K30" s="9" t="s">
-        <v>588</v>
-      </c>
-      <c r="L30" s="10" t="s">
-        <v>589</v>
+      <c r="L30" s="9" t="s">
+        <v>544</v>
       </c>
       <c r="M30" s="10" t="s">
+        <v>545</v>
+      </c>
+      <c r="N30" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="11">
-        <v>44255</v>
-      </c>
       <c r="O30" s="11">
-        <v>44261</v>
-      </c>
-      <c r="P30" s="10">
-        <v>56597</v>
+        <v>44522</v>
+      </c>
+      <c r="P30" s="11">
+        <v>44528</v>
       </c>
       <c r="Q30" s="10">
+        <v>12466</v>
+      </c>
+      <c r="R30" s="10">
         <v>3</v>
       </c>
-      <c r="R30" s="10" t="s">
-        <v>57</v>
-      </c>
       <c r="S30" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="T30" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="T30" s="32"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
@@ -12892,32 +12844,32 @@
       <c r="I31" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K31" s="9" t="s">
-        <v>592</v>
-      </c>
-      <c r="L31" s="10" t="s">
-        <v>593</v>
+      <c r="L31" s="9" t="s">
+        <v>588</v>
       </c>
       <c r="M31" s="10" t="s">
+        <v>589</v>
+      </c>
+      <c r="N31" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N31" s="11">
-        <v>43220</v>
-      </c>
       <c r="O31" s="11">
-        <v>43227</v>
-      </c>
-      <c r="P31" s="10">
-        <v>37612</v>
+        <v>44255</v>
+      </c>
+      <c r="P31" s="11">
+        <v>44261</v>
       </c>
       <c r="Q31" s="10">
-        <v>1</v>
-      </c>
-      <c r="R31" s="10" t="s">
-        <v>13</v>
+        <v>56597</v>
+      </c>
+      <c r="R31" s="10">
+        <v>3</v>
       </c>
       <c r="S31" s="10" t="s">
-        <v>23</v>
+        <v>57</v>
+      </c>
+      <c r="T31" s="12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
@@ -12948,35 +12900,35 @@
       <c r="I32" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K32" s="9" t="s">
-        <v>622</v>
-      </c>
-      <c r="L32" s="10" t="s">
-        <v>623</v>
+      <c r="L32" s="9" t="s">
+        <v>592</v>
       </c>
       <c r="M32" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="N32" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N32" s="11">
-        <v>44462</v>
-      </c>
       <c r="O32" s="11">
-        <v>44467</v>
-      </c>
-      <c r="P32" s="10">
-        <v>27196</v>
+        <v>43220</v>
+      </c>
+      <c r="P32" s="11">
+        <v>43227</v>
       </c>
       <c r="Q32" s="10">
-        <v>5</v>
-      </c>
-      <c r="R32" s="10" t="s">
-        <v>61</v>
+        <v>37612</v>
+      </c>
+      <c r="R32" s="10">
+        <v>1</v>
       </c>
       <c r="S32" s="10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+      <c r="T32" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>94</v>
       </c>
@@ -13004,8 +12956,35 @@
       <c r="I33" s="10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L33" s="9" t="s">
+        <v>622</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>623</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="O33" s="11">
+        <v>44462</v>
+      </c>
+      <c r="P33" s="11">
+        <v>44467</v>
+      </c>
+      <c r="Q33" s="10">
+        <v>27196</v>
+      </c>
+      <c r="R33" s="10">
+        <v>5</v>
+      </c>
+      <c r="S33" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="T33" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>96</v>
       </c>
@@ -13034,7 +13013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>98</v>
       </c>
@@ -13063,7 +13042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>100</v>
       </c>
@@ -13092,7 +13071,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>102</v>
       </c>
@@ -13121,7 +13100,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>104</v>
       </c>
@@ -13150,7 +13129,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>106</v>
       </c>
@@ -13179,7 +13158,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>108</v>
       </c>
@@ -13208,7 +13187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
         <v>110</v>
       </c>
@@ -13237,7 +13216,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>113</v>
       </c>
@@ -13266,7 +13245,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>115</v>
       </c>
@@ -13295,7 +13274,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="9" t="s">
         <v>117</v>
       </c>
@@ -13324,7 +13303,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
         <v>119</v>
       </c>
@@ -13353,7 +13332,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
         <v>121</v>
       </c>
@@ -13382,7 +13361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
         <v>123</v>
       </c>
@@ -13411,7 +13390,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
         <v>125</v>
       </c>
@@ -20847,12 +20826,12 @@
       <c r="I2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="26" t="s">
         <v>631</v>
       </c>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="24"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -20882,10 +20861,10 @@
       <c r="I3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="27"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="31"/>
       <c r="O3" s="17"/>
       <c r="P3" s="17"/>
       <c r="Q3" s="17"/>
@@ -20924,10 +20903,10 @@
       <c r="I4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="31"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -20957,10 +20936,10 @@
       <c r="I5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="25"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
@@ -20990,10 +20969,10 @@
       <c r="I6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="25"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="27"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
+      <c r="N6" s="31"/>
     </row>
     <row r="7" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
@@ -21023,10 +21002,10 @@
       <c r="I7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="28"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="29"/>
-      <c r="N7" s="30"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="34"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
@@ -21123,12 +21102,6 @@
       <c r="M10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N10" s="32"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="32"/>
-      <c r="R10" s="32"/>
-      <c r="S10" s="32"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -21170,12 +21143,6 @@
         <f>"=North"</f>
         <v>=North</v>
       </c>
-      <c r="N11" s="32"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="32"/>
-      <c r="Q11" s="32"/>
-      <c r="R11" s="32"/>
-      <c r="S11" s="32"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
@@ -21205,15 +21172,6 @@
       <c r="I12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K12" s="32"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="32"/>
-      <c r="N12" s="32"/>
-      <c r="O12" s="32"/>
-      <c r="P12" s="32"/>
-      <c r="Q12" s="32"/>
-      <c r="R12" s="32"/>
-      <c r="S12" s="32"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
@@ -21243,15 +21201,6 @@
       <c r="I13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="32"/>
-      <c r="N13" s="32"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="32"/>
-      <c r="Q13" s="32"/>
-      <c r="R13" s="32"/>
-      <c r="S13" s="32"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -21281,17 +21230,8 @@
       <c r="I14" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="32"/>
-      <c r="L14" s="32"/>
-      <c r="M14" s="32"/>
-      <c r="N14" s="32"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="32"/>
-      <c r="Q14" s="32"/>
-      <c r="R14" s="32"/>
-      <c r="S14" s="32"/>
-    </row>
-    <row r="15" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>52</v>
       </c>
@@ -21319,35 +21259,8 @@
       <c r="I15" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="P15" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="S15" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>55</v>
       </c>
@@ -21375,32 +21288,32 @@
       <c r="I16" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K16" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="N16" s="11">
-        <v>43173</v>
-      </c>
-      <c r="O16" s="11">
-        <v>43175</v>
-      </c>
-      <c r="P16" s="10">
-        <v>33435</v>
-      </c>
-      <c r="Q16" s="10">
+      <c r="K16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="N16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="S16" s="12" t="s">
-        <v>14</v>
+      <c r="O16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="S16" s="4" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
@@ -21432,22 +21345,22 @@
         <v>19</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>538</v>
+        <v>68</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>539</v>
+        <v>69</v>
       </c>
       <c r="M17" s="10" t="s">
         <v>35</v>
       </c>
       <c r="N17" s="11">
-        <v>43192</v>
+        <v>43173</v>
       </c>
       <c r="O17" s="11">
-        <v>43195</v>
+        <v>43175</v>
       </c>
       <c r="P17" s="10">
-        <v>41029</v>
+        <v>33435</v>
       </c>
       <c r="Q17" s="10">
         <v>3</v>
@@ -21487,15 +21400,33 @@
       <c r="I18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
-      <c r="R18" s="32"/>
-      <c r="S18" s="32"/>
+      <c r="K18" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>539</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="N18" s="11">
+        <v>43192</v>
+      </c>
+      <c r="O18" s="11">
+        <v>43195</v>
+      </c>
+      <c r="P18" s="10">
+        <v>41029</v>
+      </c>
+      <c r="Q18" s="10">
+        <v>3</v>
+      </c>
+      <c r="R18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="S18" s="12" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -21525,15 +21456,6 @@
       <c r="I19" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
@@ -29739,12 +29661,12 @@
       <c r="I2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="26" t="s">
         <v>632</v>
       </c>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="24"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -29774,10 +29696,10 @@
       <c r="I3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="27"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="31"/>
     </row>
     <row r="4" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -29807,10 +29729,10 @@
       <c r="I4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="31"/>
       <c r="O4" s="17"/>
       <c r="P4" s="17"/>
       <c r="Q4" s="17"/>
@@ -29849,10 +29771,10 @@
       <c r="I5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="25"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
@@ -29882,10 +29804,10 @@
       <c r="I6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="28"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="30"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="34"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
@@ -30077,7 +29999,7 @@
       <c r="I12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="L12" s="36" t="str">
+      <c r="L12" s="25" t="str">
         <f>"=Debit Card"</f>
         <v>=Debit Card</v>
       </c>
@@ -30107,19 +30029,9 @@
       <c r="H13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="32"/>
-      <c r="N13" s="32"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="32"/>
-      <c r="Q13" s="32"/>
-      <c r="R13" s="32"/>
-      <c r="S13" s="32"/>
+      <c r="I13" s="24" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="14" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -30146,19 +30058,18 @@
       <c r="H14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I14" s="35" t="s">
+      <c r="I14" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J14" s="32"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="33"/>
-      <c r="O14" s="31"/>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
-      <c r="R14" s="31"/>
-      <c r="S14" s="31"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
@@ -30185,19 +30096,11 @@
       <c r="H15" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I15" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J15" s="32"/>
-      <c r="K15" s="32"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="32"/>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="32"/>
-      <c r="Q15" s="32"/>
-      <c r="R15" s="32"/>
-      <c r="S15" s="32"/>
+      <c r="I15" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
@@ -30224,21 +30127,13 @@
       <c r="H16" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I16" s="35" t="s">
+      <c r="I16" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
-      <c r="P16" s="32"/>
-      <c r="Q16" s="32"/>
-      <c r="R16" s="32"/>
-      <c r="S16" s="32"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>58</v>
       </c>
@@ -30263,21 +30158,13 @@
       <c r="H17" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I17" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" s="32"/>
-      <c r="K17" s="32"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="32"/>
-      <c r="N17" s="34"/>
-      <c r="O17" s="34"/>
-      <c r="P17" s="32"/>
-      <c r="Q17" s="32"/>
-      <c r="R17" s="32"/>
-      <c r="S17" s="32"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I17" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>62</v>
       </c>
@@ -30302,21 +30189,13 @@
       <c r="H18" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I18" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="32"/>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
-      <c r="P18" s="32"/>
-      <c r="Q18" s="32"/>
-      <c r="R18" s="32"/>
-      <c r="S18" s="32"/>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I18" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -30341,21 +30220,13 @@
       <c r="H19" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I19" s="35" t="s">
+      <c r="I19" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="34"/>
-      <c r="O19" s="34"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>66</v>
       </c>
@@ -30380,21 +30251,13 @@
       <c r="H20" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I20" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J20" s="32"/>
-      <c r="K20" s="32"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="32"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
-      <c r="P20" s="32"/>
-      <c r="Q20" s="32"/>
-      <c r="R20" s="32"/>
-      <c r="S20" s="32"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I20" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N20" s="23"/>
+      <c r="O20" s="23"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>68</v>
       </c>
@@ -30419,21 +30282,13 @@
       <c r="H21" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="35" t="s">
+      <c r="I21" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="34"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>70</v>
       </c>
@@ -30458,21 +30313,13 @@
       <c r="H22" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="35" t="s">
+      <c r="I22" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J22" s="32"/>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="32"/>
-      <c r="Q22" s="32"/>
-      <c r="R22" s="32"/>
-      <c r="S22" s="32"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N22" s="23"/>
+      <c r="O22" s="23"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>72</v>
       </c>
@@ -30497,21 +30344,13 @@
       <c r="H23" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I23" s="35" t="s">
+      <c r="I23" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J23" s="32"/>
-      <c r="K23" s="32"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="34"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="32"/>
-      <c r="R23" s="32"/>
-      <c r="S23" s="32"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N23" s="23"/>
+      <c r="O23" s="23"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>74</v>
       </c>
@@ -30536,21 +30375,13 @@
       <c r="H24" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I24" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="34"/>
-      <c r="P24" s="32"/>
-      <c r="Q24" s="32"/>
-      <c r="R24" s="32"/>
-      <c r="S24" s="32"/>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I24" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N24" s="23"/>
+      <c r="O24" s="23"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>76</v>
       </c>
@@ -30575,21 +30406,13 @@
       <c r="H25" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I25" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="N25" s="34"/>
-      <c r="O25" s="34"/>
-      <c r="P25" s="32"/>
-      <c r="Q25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I25" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>79</v>
       </c>
@@ -30614,21 +30437,13 @@
       <c r="H26" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I26" s="35" t="s">
+      <c r="I26" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="34"/>
-      <c r="O26" s="34"/>
-      <c r="P26" s="32"/>
-      <c r="Q26" s="32"/>
-      <c r="R26" s="32"/>
-      <c r="S26" s="32"/>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>82</v>
       </c>
@@ -30653,21 +30468,13 @@
       <c r="H27" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I27" s="35" t="s">
+      <c r="I27" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="34"/>
-      <c r="O27" s="34"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="32"/>
-      <c r="R27" s="32"/>
-      <c r="S27" s="32"/>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>84</v>
       </c>
@@ -30692,21 +30499,13 @@
       <c r="H28" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28" s="32"/>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
-      <c r="P28" s="32"/>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I28" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>86</v>
       </c>
@@ -30731,21 +30530,13 @@
       <c r="H29" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I29" s="35" t="s">
+      <c r="I29" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J29" s="32"/>
-      <c r="K29" s="32"/>
-      <c r="L29" s="32"/>
-      <c r="M29" s="32"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="32"/>
-      <c r="Q29" s="32"/>
-      <c r="R29" s="32"/>
-      <c r="S29" s="32"/>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>88</v>
       </c>
@@ -30770,21 +30561,13 @@
       <c r="H30" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I30" s="35" t="s">
+      <c r="I30" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="34"/>
-      <c r="O30" s="34"/>
-      <c r="P30" s="32"/>
-      <c r="Q30" s="32"/>
-      <c r="R30" s="32"/>
-      <c r="S30" s="32"/>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>90</v>
       </c>
@@ -30809,21 +30592,13 @@
       <c r="H31" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I31" s="35" t="s">
+      <c r="I31" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J31" s="32"/>
-      <c r="K31" s="32"/>
-      <c r="L31" s="32"/>
-      <c r="M31" s="32"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="32"/>
-      <c r="Q31" s="32"/>
-      <c r="R31" s="32"/>
-      <c r="S31" s="32"/>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>92</v>
       </c>
@@ -30848,21 +30623,13 @@
       <c r="H32" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I32" s="35" t="s">
+      <c r="I32" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="32"/>
-      <c r="K32" s="32"/>
-      <c r="L32" s="32"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="34"/>
-      <c r="O32" s="34"/>
-      <c r="P32" s="32"/>
-      <c r="Q32" s="32"/>
-      <c r="R32" s="32"/>
-      <c r="S32" s="32"/>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>94</v>
       </c>
@@ -30887,21 +30654,13 @@
       <c r="H33" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I33" s="35" t="s">
+      <c r="I33" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J33" s="32"/>
-      <c r="K33" s="32"/>
-      <c r="L33" s="32"/>
-      <c r="M33" s="32"/>
-      <c r="N33" s="34"/>
-      <c r="O33" s="34"/>
-      <c r="P33" s="32"/>
-      <c r="Q33" s="32"/>
-      <c r="R33" s="32"/>
-      <c r="S33" s="32"/>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N33" s="23"/>
+      <c r="O33" s="23"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>96</v>
       </c>
@@ -30926,21 +30685,13 @@
       <c r="H34" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I34" s="35" t="s">
+      <c r="I34" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="32"/>
-      <c r="K34" s="32"/>
-      <c r="L34" s="32"/>
-      <c r="M34" s="32"/>
-      <c r="N34" s="34"/>
-      <c r="O34" s="34"/>
-      <c r="P34" s="32"/>
-      <c r="Q34" s="32"/>
-      <c r="R34" s="32"/>
-      <c r="S34" s="32"/>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N34" s="23"/>
+      <c r="O34" s="23"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>98</v>
       </c>
@@ -30965,21 +30716,13 @@
       <c r="H35" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I35" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J35" s="32"/>
-      <c r="K35" s="32"/>
-      <c r="L35" s="32"/>
-      <c r="M35" s="32"/>
-      <c r="N35" s="34"/>
-      <c r="O35" s="34"/>
-      <c r="P35" s="32"/>
-      <c r="Q35" s="32"/>
-      <c r="R35" s="32"/>
-      <c r="S35" s="32"/>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I35" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>100</v>
       </c>
@@ -31004,21 +30747,13 @@
       <c r="H36" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="35" t="s">
+      <c r="I36" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J36" s="32"/>
-      <c r="K36" s="32"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="32"/>
-      <c r="N36" s="34"/>
-      <c r="O36" s="34"/>
-      <c r="P36" s="32"/>
-      <c r="Q36" s="32"/>
-      <c r="R36" s="32"/>
-      <c r="S36" s="32"/>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N36" s="23"/>
+      <c r="O36" s="23"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>102</v>
       </c>
@@ -31043,21 +30778,13 @@
       <c r="H37" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I37" s="35" t="s">
+      <c r="I37" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J37" s="32"/>
-      <c r="K37" s="32"/>
-      <c r="L37" s="32"/>
-      <c r="M37" s="32"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
-      <c r="P37" s="32"/>
-      <c r="Q37" s="32"/>
-      <c r="R37" s="32"/>
-      <c r="S37" s="32"/>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>104</v>
       </c>
@@ -31082,21 +30809,13 @@
       <c r="H38" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I38" s="35" t="s">
+      <c r="I38" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J38" s="32"/>
-      <c r="K38" s="32"/>
-      <c r="L38" s="32"/>
-      <c r="M38" s="32"/>
-      <c r="N38" s="34"/>
-      <c r="O38" s="34"/>
-      <c r="P38" s="32"/>
-      <c r="Q38" s="32"/>
-      <c r="R38" s="32"/>
-      <c r="S38" s="32"/>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N38" s="23"/>
+      <c r="O38" s="23"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>106</v>
       </c>
@@ -31121,21 +30840,13 @@
       <c r="H39" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I39" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J39" s="32"/>
-      <c r="K39" s="32"/>
-      <c r="L39" s="32"/>
-      <c r="M39" s="32"/>
-      <c r="N39" s="34"/>
-      <c r="O39" s="34"/>
-      <c r="P39" s="32"/>
-      <c r="Q39" s="32"/>
-      <c r="R39" s="32"/>
-      <c r="S39" s="32"/>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I39" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N39" s="23"/>
+      <c r="O39" s="23"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>108</v>
       </c>
@@ -31160,21 +30871,13 @@
       <c r="H40" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I40" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J40" s="32"/>
-      <c r="K40" s="32"/>
-      <c r="L40" s="32"/>
-      <c r="M40" s="32"/>
-      <c r="N40" s="34"/>
-      <c r="O40" s="34"/>
-      <c r="P40" s="32"/>
-      <c r="Q40" s="32"/>
-      <c r="R40" s="32"/>
-      <c r="S40" s="32"/>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I40" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
         <v>110</v>
       </c>
@@ -31199,21 +30902,13 @@
       <c r="H41" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I41" s="35" t="s">
+      <c r="I41" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J41" s="32"/>
-      <c r="K41" s="32"/>
-      <c r="L41" s="32"/>
-      <c r="M41" s="32"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
-      <c r="P41" s="32"/>
-      <c r="Q41" s="32"/>
-      <c r="R41" s="32"/>
-      <c r="S41" s="32"/>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>113</v>
       </c>
@@ -31238,21 +30933,13 @@
       <c r="H42" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I42" s="35" t="s">
+      <c r="I42" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="32"/>
-      <c r="N42" s="34"/>
-      <c r="O42" s="34"/>
-      <c r="P42" s="32"/>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="32"/>
-      <c r="S42" s="32"/>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>115</v>
       </c>
@@ -31277,21 +30964,13 @@
       <c r="H43" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I43" s="35" t="s">
+      <c r="I43" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J43" s="32"/>
-      <c r="K43" s="32"/>
-      <c r="L43" s="32"/>
-      <c r="M43" s="32"/>
-      <c r="N43" s="34"/>
-      <c r="O43" s="34"/>
-      <c r="P43" s="32"/>
-      <c r="Q43" s="32"/>
-      <c r="R43" s="32"/>
-      <c r="S43" s="32"/>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N43" s="23"/>
+      <c r="O43" s="23"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="9" t="s">
         <v>117</v>
       </c>
@@ -31316,21 +30995,13 @@
       <c r="H44" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I44" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J44" s="32"/>
-      <c r="K44" s="32"/>
-      <c r="L44" s="32"/>
-      <c r="M44" s="32"/>
-      <c r="N44" s="34"/>
-      <c r="O44" s="34"/>
-      <c r="P44" s="32"/>
-      <c r="Q44" s="32"/>
-      <c r="R44" s="32"/>
-      <c r="S44" s="32"/>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I44" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N44" s="23"/>
+      <c r="O44" s="23"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
         <v>119</v>
       </c>
@@ -31355,21 +31026,13 @@
       <c r="H45" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I45" s="35" t="s">
+      <c r="I45" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J45" s="32"/>
-      <c r="K45" s="32"/>
-      <c r="L45" s="32"/>
-      <c r="M45" s="32"/>
-      <c r="N45" s="34"/>
-      <c r="O45" s="34"/>
-      <c r="P45" s="32"/>
-      <c r="Q45" s="32"/>
-      <c r="R45" s="32"/>
-      <c r="S45" s="32"/>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N45" s="23"/>
+      <c r="O45" s="23"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
         <v>121</v>
       </c>
@@ -31394,21 +31057,13 @@
       <c r="H46" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I46" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J46" s="32"/>
-      <c r="K46" s="32"/>
-      <c r="L46" s="32"/>
-      <c r="M46" s="32"/>
-      <c r="N46" s="34"/>
-      <c r="O46" s="34"/>
-      <c r="P46" s="32"/>
-      <c r="Q46" s="32"/>
-      <c r="R46" s="32"/>
-      <c r="S46" s="32"/>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I46" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
         <v>123</v>
       </c>
@@ -31433,21 +31088,13 @@
       <c r="H47" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I47" s="35" t="s">
+      <c r="I47" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J47" s="32"/>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
-      <c r="N47" s="34"/>
-      <c r="O47" s="34"/>
-      <c r="P47" s="32"/>
-      <c r="Q47" s="32"/>
-      <c r="R47" s="32"/>
-      <c r="S47" s="32"/>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N47" s="23"/>
+      <c r="O47" s="23"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
         <v>125</v>
       </c>
@@ -31472,21 +31119,13 @@
       <c r="H48" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I48" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="32"/>
-      <c r="N48" s="34"/>
-      <c r="O48" s="34"/>
-      <c r="P48" s="32"/>
-      <c r="Q48" s="32"/>
-      <c r="R48" s="32"/>
-      <c r="S48" s="32"/>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I48" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N48" s="23"/>
+      <c r="O48" s="23"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="9" t="s">
         <v>127</v>
       </c>
@@ -31511,21 +31150,13 @@
       <c r="H49" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I49" s="35" t="s">
+      <c r="I49" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J49" s="32"/>
-      <c r="K49" s="32"/>
-      <c r="L49" s="32"/>
-      <c r="M49" s="32"/>
-      <c r="N49" s="34"/>
-      <c r="O49" s="34"/>
-      <c r="P49" s="32"/>
-      <c r="Q49" s="32"/>
-      <c r="R49" s="32"/>
-      <c r="S49" s="32"/>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N49" s="23"/>
+      <c r="O49" s="23"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -31550,21 +31181,13 @@
       <c r="H50" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I50" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J50" s="32"/>
-      <c r="K50" s="32"/>
-      <c r="L50" s="32"/>
-      <c r="M50" s="32"/>
-      <c r="N50" s="34"/>
-      <c r="O50" s="34"/>
-      <c r="P50" s="32"/>
-      <c r="Q50" s="32"/>
-      <c r="R50" s="32"/>
-      <c r="S50" s="32"/>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I50" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N50" s="23"/>
+      <c r="O50" s="23"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
         <v>131</v>
       </c>
@@ -31589,21 +31212,13 @@
       <c r="H51" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I51" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J51" s="32"/>
-      <c r="K51" s="32"/>
-      <c r="L51" s="32"/>
-      <c r="M51" s="32"/>
-      <c r="N51" s="34"/>
-      <c r="O51" s="34"/>
-      <c r="P51" s="32"/>
-      <c r="Q51" s="32"/>
-      <c r="R51" s="32"/>
-      <c r="S51" s="32"/>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I51" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N51" s="23"/>
+      <c r="O51" s="23"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
         <v>133</v>
       </c>
@@ -31628,21 +31243,13 @@
       <c r="H52" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I52" s="35" t="s">
+      <c r="I52" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J52" s="32"/>
-      <c r="K52" s="32"/>
-      <c r="L52" s="32"/>
-      <c r="M52" s="32"/>
-      <c r="N52" s="34"/>
-      <c r="O52" s="34"/>
-      <c r="P52" s="32"/>
-      <c r="Q52" s="32"/>
-      <c r="R52" s="32"/>
-      <c r="S52" s="32"/>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
         <v>135</v>
       </c>
@@ -31667,21 +31274,13 @@
       <c r="H53" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I53" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J53" s="32"/>
-      <c r="K53" s="32"/>
-      <c r="L53" s="32"/>
-      <c r="M53" s="32"/>
-      <c r="N53" s="34"/>
-      <c r="O53" s="34"/>
-      <c r="P53" s="32"/>
-      <c r="Q53" s="32"/>
-      <c r="R53" s="32"/>
-      <c r="S53" s="32"/>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I53" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N53" s="23"/>
+      <c r="O53" s="23"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
         <v>137</v>
       </c>
@@ -31706,21 +31305,13 @@
       <c r="H54" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I54" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J54" s="32"/>
-      <c r="K54" s="32"/>
-      <c r="L54" s="32"/>
-      <c r="M54" s="32"/>
-      <c r="N54" s="34"/>
-      <c r="O54" s="34"/>
-      <c r="P54" s="32"/>
-      <c r="Q54" s="32"/>
-      <c r="R54" s="32"/>
-      <c r="S54" s="32"/>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I54" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N54" s="23"/>
+      <c r="O54" s="23"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
         <v>139</v>
       </c>
@@ -31745,21 +31336,13 @@
       <c r="H55" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I55" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J55" s="32"/>
-      <c r="K55" s="32"/>
-      <c r="L55" s="32"/>
-      <c r="M55" s="32"/>
-      <c r="N55" s="34"/>
-      <c r="O55" s="34"/>
-      <c r="P55" s="32"/>
-      <c r="Q55" s="32"/>
-      <c r="R55" s="32"/>
-      <c r="S55" s="32"/>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I55" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N55" s="23"/>
+      <c r="O55" s="23"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
         <v>141</v>
       </c>
@@ -31784,21 +31367,13 @@
       <c r="H56" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I56" s="35" t="s">
+      <c r="I56" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J56" s="32"/>
-      <c r="K56" s="32"/>
-      <c r="L56" s="32"/>
-      <c r="M56" s="32"/>
-      <c r="N56" s="34"/>
-      <c r="O56" s="34"/>
-      <c r="P56" s="32"/>
-      <c r="Q56" s="32"/>
-      <c r="R56" s="32"/>
-      <c r="S56" s="32"/>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N56" s="23"/>
+      <c r="O56" s="23"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
         <v>143</v>
       </c>
@@ -31823,21 +31398,13 @@
       <c r="H57" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I57" s="35" t="s">
+      <c r="I57" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J57" s="32"/>
-      <c r="K57" s="32"/>
-      <c r="L57" s="32"/>
-      <c r="M57" s="32"/>
-      <c r="N57" s="34"/>
-      <c r="O57" s="34"/>
-      <c r="P57" s="32"/>
-      <c r="Q57" s="32"/>
-      <c r="R57" s="32"/>
-      <c r="S57" s="32"/>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N57" s="23"/>
+      <c r="O57" s="23"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
         <v>145</v>
       </c>
@@ -31862,21 +31429,13 @@
       <c r="H58" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I58" s="35" t="s">
+      <c r="I58" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J58" s="32"/>
-      <c r="K58" s="32"/>
-      <c r="L58" s="32"/>
-      <c r="M58" s="32"/>
-      <c r="N58" s="34"/>
-      <c r="O58" s="34"/>
-      <c r="P58" s="32"/>
-      <c r="Q58" s="32"/>
-      <c r="R58" s="32"/>
-      <c r="S58" s="32"/>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N58" s="23"/>
+      <c r="O58" s="23"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
         <v>147</v>
       </c>
@@ -31901,21 +31460,13 @@
       <c r="H59" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I59" s="35" t="s">
+      <c r="I59" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J59" s="32"/>
-      <c r="K59" s="32"/>
-      <c r="L59" s="32"/>
-      <c r="M59" s="32"/>
-      <c r="N59" s="34"/>
-      <c r="O59" s="34"/>
-      <c r="P59" s="32"/>
-      <c r="Q59" s="32"/>
-      <c r="R59" s="32"/>
-      <c r="S59" s="32"/>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N59" s="23"/>
+      <c r="O59" s="23"/>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
         <v>149</v>
       </c>
@@ -31940,21 +31491,13 @@
       <c r="H60" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I60" s="35" t="s">
+      <c r="I60" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J60" s="32"/>
-      <c r="K60" s="32"/>
-      <c r="L60" s="32"/>
-      <c r="M60" s="32"/>
-      <c r="N60" s="34"/>
-      <c r="O60" s="34"/>
-      <c r="P60" s="32"/>
-      <c r="Q60" s="32"/>
-      <c r="R60" s="32"/>
-      <c r="S60" s="32"/>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N60" s="23"/>
+      <c r="O60" s="23"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>152</v>
       </c>
@@ -31979,21 +31522,13 @@
       <c r="H61" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I61" s="35" t="s">
+      <c r="I61" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J61" s="32"/>
-      <c r="K61" s="32"/>
-      <c r="L61" s="32"/>
-      <c r="M61" s="32"/>
-      <c r="N61" s="34"/>
-      <c r="O61" s="34"/>
-      <c r="P61" s="32"/>
-      <c r="Q61" s="32"/>
-      <c r="R61" s="32"/>
-      <c r="S61" s="32"/>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N61" s="23"/>
+      <c r="O61" s="23"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
         <v>154</v>
       </c>
@@ -32018,21 +31553,13 @@
       <c r="H62" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I62" s="35" t="s">
+      <c r="I62" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J62" s="32"/>
-      <c r="K62" s="32"/>
-      <c r="L62" s="32"/>
-      <c r="M62" s="32"/>
-      <c r="N62" s="34"/>
-      <c r="O62" s="34"/>
-      <c r="P62" s="32"/>
-      <c r="Q62" s="32"/>
-      <c r="R62" s="32"/>
-      <c r="S62" s="32"/>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N62" s="23"/>
+      <c r="O62" s="23"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
         <v>156</v>
       </c>
@@ -32057,21 +31584,13 @@
       <c r="H63" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I63" s="35" t="s">
+      <c r="I63" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J63" s="32"/>
-      <c r="K63" s="32"/>
-      <c r="L63" s="32"/>
-      <c r="M63" s="32"/>
-      <c r="N63" s="34"/>
-      <c r="O63" s="34"/>
-      <c r="P63" s="32"/>
-      <c r="Q63" s="32"/>
-      <c r="R63" s="32"/>
-      <c r="S63" s="32"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N63" s="23"/>
+      <c r="O63" s="23"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>158</v>
       </c>
@@ -32096,21 +31615,13 @@
       <c r="H64" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I64" s="35" t="s">
+      <c r="I64" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J64" s="32"/>
-      <c r="K64" s="32"/>
-      <c r="L64" s="32"/>
-      <c r="M64" s="32"/>
-      <c r="N64" s="34"/>
-      <c r="O64" s="34"/>
-      <c r="P64" s="32"/>
-      <c r="Q64" s="32"/>
-      <c r="R64" s="32"/>
-      <c r="S64" s="32"/>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N64" s="23"/>
+      <c r="O64" s="23"/>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="9" t="s">
         <v>160</v>
       </c>
@@ -32135,21 +31646,13 @@
       <c r="H65" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I65" s="35" t="s">
+      <c r="I65" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J65" s="32"/>
-      <c r="K65" s="32"/>
-      <c r="L65" s="32"/>
-      <c r="M65" s="32"/>
-      <c r="N65" s="34"/>
-      <c r="O65" s="34"/>
-      <c r="P65" s="32"/>
-      <c r="Q65" s="32"/>
-      <c r="R65" s="32"/>
-      <c r="S65" s="32"/>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N65" s="23"/>
+      <c r="O65" s="23"/>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="9" t="s">
         <v>162</v>
       </c>
@@ -32174,21 +31677,13 @@
       <c r="H66" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I66" s="35" t="s">
+      <c r="I66" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J66" s="32"/>
-      <c r="K66" s="32"/>
-      <c r="L66" s="32"/>
-      <c r="M66" s="32"/>
-      <c r="N66" s="34"/>
-      <c r="O66" s="34"/>
-      <c r="P66" s="32"/>
-      <c r="Q66" s="32"/>
-      <c r="R66" s="32"/>
-      <c r="S66" s="32"/>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N66" s="23"/>
+      <c r="O66" s="23"/>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="9" t="s">
         <v>164</v>
       </c>
@@ -32213,21 +31708,13 @@
       <c r="H67" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I67" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J67" s="32"/>
-      <c r="K67" s="32"/>
-      <c r="L67" s="32"/>
-      <c r="M67" s="32"/>
-      <c r="N67" s="34"/>
-      <c r="O67" s="34"/>
-      <c r="P67" s="32"/>
-      <c r="Q67" s="32"/>
-      <c r="R67" s="32"/>
-      <c r="S67" s="32"/>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I67" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N67" s="23"/>
+      <c r="O67" s="23"/>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
         <v>166</v>
       </c>
@@ -32252,21 +31739,13 @@
       <c r="H68" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I68" s="35" t="s">
+      <c r="I68" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J68" s="32"/>
-      <c r="K68" s="32"/>
-      <c r="L68" s="32"/>
-      <c r="M68" s="32"/>
-      <c r="N68" s="34"/>
-      <c r="O68" s="34"/>
-      <c r="P68" s="32"/>
-      <c r="Q68" s="32"/>
-      <c r="R68" s="32"/>
-      <c r="S68" s="32"/>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N68" s="23"/>
+      <c r="O68" s="23"/>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="9" t="s">
         <v>168</v>
       </c>
@@ -32291,21 +31770,13 @@
       <c r="H69" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I69" s="35" t="s">
+      <c r="I69" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J69" s="32"/>
-      <c r="K69" s="32"/>
-      <c r="L69" s="32"/>
-      <c r="M69" s="32"/>
-      <c r="N69" s="34"/>
-      <c r="O69" s="34"/>
-      <c r="P69" s="32"/>
-      <c r="Q69" s="32"/>
-      <c r="R69" s="32"/>
-      <c r="S69" s="32"/>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N69" s="23"/>
+      <c r="O69" s="23"/>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="9" t="s">
         <v>170</v>
       </c>
@@ -32330,21 +31801,13 @@
       <c r="H70" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I70" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J70" s="32"/>
-      <c r="K70" s="32"/>
-      <c r="L70" s="32"/>
-      <c r="M70" s="32"/>
-      <c r="N70" s="34"/>
-      <c r="O70" s="34"/>
-      <c r="P70" s="32"/>
-      <c r="Q70" s="32"/>
-      <c r="R70" s="32"/>
-      <c r="S70" s="32"/>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I70" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="N70" s="23"/>
+      <c r="O70" s="23"/>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="9" t="s">
         <v>172</v>
       </c>
@@ -32369,21 +31832,13 @@
       <c r="H71" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I71" s="35" t="s">
+      <c r="I71" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J71" s="32"/>
-      <c r="K71" s="32"/>
-      <c r="L71" s="32"/>
-      <c r="M71" s="32"/>
-      <c r="N71" s="34"/>
-      <c r="O71" s="34"/>
-      <c r="P71" s="32"/>
-      <c r="Q71" s="32"/>
-      <c r="R71" s="32"/>
-      <c r="S71" s="32"/>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N71" s="23"/>
+      <c r="O71" s="23"/>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="9" t="s">
         <v>174</v>
       </c>
@@ -32408,21 +31863,13 @@
       <c r="H72" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I72" s="35" t="s">
+      <c r="I72" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J72" s="32"/>
-      <c r="K72" s="32"/>
-      <c r="L72" s="32"/>
-      <c r="M72" s="32"/>
-      <c r="N72" s="34"/>
-      <c r="O72" s="34"/>
-      <c r="P72" s="32"/>
-      <c r="Q72" s="32"/>
-      <c r="R72" s="32"/>
-      <c r="S72" s="32"/>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N72" s="23"/>
+      <c r="O72" s="23"/>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="9" t="s">
         <v>176</v>
       </c>
@@ -32447,21 +31894,13 @@
       <c r="H73" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I73" s="35" t="s">
+      <c r="I73" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J73" s="32"/>
-      <c r="K73" s="32"/>
-      <c r="L73" s="32"/>
-      <c r="M73" s="32"/>
-      <c r="N73" s="34"/>
-      <c r="O73" s="34"/>
-      <c r="P73" s="32"/>
-      <c r="Q73" s="32"/>
-      <c r="R73" s="32"/>
-      <c r="S73" s="32"/>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N73" s="23"/>
+      <c r="O73" s="23"/>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="9" t="s">
         <v>178</v>
       </c>
@@ -32486,21 +31925,13 @@
       <c r="H74" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I74" s="35" t="s">
+      <c r="I74" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J74" s="32"/>
-      <c r="K74" s="32"/>
-      <c r="L74" s="32"/>
-      <c r="M74" s="32"/>
-      <c r="N74" s="34"/>
-      <c r="O74" s="34"/>
-      <c r="P74" s="32"/>
-      <c r="Q74" s="32"/>
-      <c r="R74" s="32"/>
-      <c r="S74" s="32"/>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="N74" s="23"/>
+      <c r="O74" s="23"/>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75" s="9" t="s">
         <v>180</v>
       </c>
@@ -32525,21 +31956,11 @@
       <c r="H75" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I75" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J75" s="32"/>
-      <c r="K75" s="32"/>
-      <c r="L75" s="32"/>
-      <c r="M75" s="32"/>
-      <c r="N75" s="32"/>
-      <c r="O75" s="32"/>
-      <c r="P75" s="32"/>
-      <c r="Q75" s="32"/>
-      <c r="R75" s="32"/>
-      <c r="S75" s="32"/>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I75" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76" s="9" t="s">
         <v>182</v>
       </c>
@@ -32564,21 +31985,11 @@
       <c r="H76" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I76" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J76" s="32"/>
-      <c r="K76" s="32"/>
-      <c r="L76" s="32"/>
-      <c r="M76" s="32"/>
-      <c r="N76" s="32"/>
-      <c r="O76" s="32"/>
-      <c r="P76" s="32"/>
-      <c r="Q76" s="32"/>
-      <c r="R76" s="32"/>
-      <c r="S76" s="32"/>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I76" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77" s="9" t="s">
         <v>184</v>
       </c>
@@ -32603,21 +32014,11 @@
       <c r="H77" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I77" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J77" s="32"/>
-      <c r="K77" s="32"/>
-      <c r="L77" s="32"/>
-      <c r="M77" s="32"/>
-      <c r="N77" s="32"/>
-      <c r="O77" s="32"/>
-      <c r="P77" s="32"/>
-      <c r="Q77" s="32"/>
-      <c r="R77" s="32"/>
-      <c r="S77" s="32"/>
-    </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I77" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="9" t="s">
         <v>186</v>
       </c>
@@ -32642,21 +32043,11 @@
       <c r="H78" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I78" s="35" t="s">
+      <c r="I78" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J78" s="32"/>
-      <c r="K78" s="32"/>
-      <c r="L78" s="32"/>
-      <c r="M78" s="32"/>
-      <c r="N78" s="32"/>
-      <c r="O78" s="32"/>
-      <c r="P78" s="32"/>
-      <c r="Q78" s="32"/>
-      <c r="R78" s="32"/>
-      <c r="S78" s="32"/>
-    </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79" s="9" t="s">
         <v>188</v>
       </c>
@@ -32681,21 +32072,11 @@
       <c r="H79" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I79" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J79" s="32"/>
-      <c r="K79" s="32"/>
-      <c r="L79" s="32"/>
-      <c r="M79" s="32"/>
-      <c r="N79" s="32"/>
-      <c r="O79" s="32"/>
-      <c r="P79" s="32"/>
-      <c r="Q79" s="32"/>
-      <c r="R79" s="32"/>
-      <c r="S79" s="32"/>
-    </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I79" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="9" t="s">
         <v>190</v>
       </c>
@@ -32720,21 +32101,11 @@
       <c r="H80" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I80" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J80" s="32"/>
-      <c r="K80" s="32"/>
-      <c r="L80" s="32"/>
-      <c r="M80" s="32"/>
-      <c r="N80" s="32"/>
-      <c r="O80" s="32"/>
-      <c r="P80" s="32"/>
-      <c r="Q80" s="32"/>
-      <c r="R80" s="32"/>
-      <c r="S80" s="32"/>
-    </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I80" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" s="9" t="s">
         <v>192</v>
       </c>
@@ -32759,21 +32130,11 @@
       <c r="H81" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I81" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J81" s="32"/>
-      <c r="K81" s="32"/>
-      <c r="L81" s="32"/>
-      <c r="M81" s="32"/>
-      <c r="N81" s="32"/>
-      <c r="O81" s="32"/>
-      <c r="P81" s="32"/>
-      <c r="Q81" s="32"/>
-      <c r="R81" s="32"/>
-      <c r="S81" s="32"/>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I81" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" s="9" t="s">
         <v>194</v>
       </c>
@@ -32798,21 +32159,11 @@
       <c r="H82" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I82" s="35" t="s">
+      <c r="I82" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J82" s="32"/>
-      <c r="K82" s="32"/>
-      <c r="L82" s="32"/>
-      <c r="M82" s="32"/>
-      <c r="N82" s="32"/>
-      <c r="O82" s="32"/>
-      <c r="P82" s="32"/>
-      <c r="Q82" s="32"/>
-      <c r="R82" s="32"/>
-      <c r="S82" s="32"/>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83" s="9" t="s">
         <v>196</v>
       </c>
@@ -32837,21 +32188,11 @@
       <c r="H83" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I83" s="35" t="s">
+      <c r="I83" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J83" s="32"/>
-      <c r="K83" s="32"/>
-      <c r="L83" s="32"/>
-      <c r="M83" s="32"/>
-      <c r="N83" s="32"/>
-      <c r="O83" s="32"/>
-      <c r="P83" s="32"/>
-      <c r="Q83" s="32"/>
-      <c r="R83" s="32"/>
-      <c r="S83" s="32"/>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84" s="9" t="s">
         <v>198</v>
       </c>
@@ -32876,21 +32217,11 @@
       <c r="H84" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I84" s="35" t="s">
+      <c r="I84" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J84" s="32"/>
-      <c r="K84" s="32"/>
-      <c r="L84" s="32"/>
-      <c r="M84" s="32"/>
-      <c r="N84" s="32"/>
-      <c r="O84" s="32"/>
-      <c r="P84" s="32"/>
-      <c r="Q84" s="32"/>
-      <c r="R84" s="32"/>
-      <c r="S84" s="32"/>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
         <v>200</v>
       </c>
@@ -32915,21 +32246,11 @@
       <c r="H85" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I85" s="35" t="s">
+      <c r="I85" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J85" s="32"/>
-      <c r="K85" s="32"/>
-      <c r="L85" s="32"/>
-      <c r="M85" s="32"/>
-      <c r="N85" s="32"/>
-      <c r="O85" s="32"/>
-      <c r="P85" s="32"/>
-      <c r="Q85" s="32"/>
-      <c r="R85" s="32"/>
-      <c r="S85" s="32"/>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86" s="9" t="s">
         <v>202</v>
       </c>
@@ -32954,21 +32275,11 @@
       <c r="H86" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I86" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J86" s="32"/>
-      <c r="K86" s="32"/>
-      <c r="L86" s="32"/>
-      <c r="M86" s="32"/>
-      <c r="N86" s="32"/>
-      <c r="O86" s="32"/>
-      <c r="P86" s="32"/>
-      <c r="Q86" s="32"/>
-      <c r="R86" s="32"/>
-      <c r="S86" s="32"/>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I86" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87" s="9" t="s">
         <v>204</v>
       </c>
@@ -32993,21 +32304,11 @@
       <c r="H87" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I87" s="35" t="s">
+      <c r="I87" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J87" s="32"/>
-      <c r="K87" s="32"/>
-      <c r="L87" s="32"/>
-      <c r="M87" s="32"/>
-      <c r="N87" s="32"/>
-      <c r="O87" s="32"/>
-      <c r="P87" s="32"/>
-      <c r="Q87" s="32"/>
-      <c r="R87" s="32"/>
-      <c r="S87" s="32"/>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88" s="9" t="s">
         <v>206</v>
       </c>
@@ -33032,21 +32333,11 @@
       <c r="H88" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I88" s="35" t="s">
+      <c r="I88" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J88" s="32"/>
-      <c r="K88" s="32"/>
-      <c r="L88" s="32"/>
-      <c r="M88" s="32"/>
-      <c r="N88" s="32"/>
-      <c r="O88" s="32"/>
-      <c r="P88" s="32"/>
-      <c r="Q88" s="32"/>
-      <c r="R88" s="32"/>
-      <c r="S88" s="32"/>
-    </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" s="9" t="s">
         <v>208</v>
       </c>
@@ -33071,21 +32362,11 @@
       <c r="H89" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I89" s="35" t="s">
+      <c r="I89" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J89" s="32"/>
-      <c r="K89" s="32"/>
-      <c r="L89" s="32"/>
-      <c r="M89" s="32"/>
-      <c r="N89" s="32"/>
-      <c r="O89" s="32"/>
-      <c r="P89" s="32"/>
-      <c r="Q89" s="32"/>
-      <c r="R89" s="32"/>
-      <c r="S89" s="32"/>
-    </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90" s="9" t="s">
         <v>210</v>
       </c>
@@ -33110,21 +32391,11 @@
       <c r="H90" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I90" s="35" t="s">
+      <c r="I90" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J90" s="32"/>
-      <c r="K90" s="32"/>
-      <c r="L90" s="32"/>
-      <c r="M90" s="32"/>
-      <c r="N90" s="32"/>
-      <c r="O90" s="32"/>
-      <c r="P90" s="32"/>
-      <c r="Q90" s="32"/>
-      <c r="R90" s="32"/>
-      <c r="S90" s="32"/>
-    </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91" s="9" t="s">
         <v>212</v>
       </c>
@@ -33149,21 +32420,11 @@
       <c r="H91" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I91" s="35" t="s">
+      <c r="I91" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J91" s="32"/>
-      <c r="K91" s="32"/>
-      <c r="L91" s="32"/>
-      <c r="M91" s="32"/>
-      <c r="N91" s="32"/>
-      <c r="O91" s="32"/>
-      <c r="P91" s="32"/>
-      <c r="Q91" s="32"/>
-      <c r="R91" s="32"/>
-      <c r="S91" s="32"/>
-    </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" s="9" t="s">
         <v>214</v>
       </c>
@@ -33188,21 +32449,11 @@
       <c r="H92" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I92" s="35" t="s">
+      <c r="I92" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J92" s="32"/>
-      <c r="K92" s="32"/>
-      <c r="L92" s="32"/>
-      <c r="M92" s="32"/>
-      <c r="N92" s="32"/>
-      <c r="O92" s="32"/>
-      <c r="P92" s="32"/>
-      <c r="Q92" s="32"/>
-      <c r="R92" s="32"/>
-      <c r="S92" s="32"/>
-    </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" s="9" t="s">
         <v>216</v>
       </c>
@@ -33227,21 +32478,11 @@
       <c r="H93" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I93" s="35" t="s">
+      <c r="I93" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J93" s="32"/>
-      <c r="K93" s="32"/>
-      <c r="L93" s="32"/>
-      <c r="M93" s="32"/>
-      <c r="N93" s="32"/>
-      <c r="O93" s="32"/>
-      <c r="P93" s="32"/>
-      <c r="Q93" s="32"/>
-      <c r="R93" s="32"/>
-      <c r="S93" s="32"/>
-    </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" s="9" t="s">
         <v>218</v>
       </c>
@@ -33266,21 +32507,11 @@
       <c r="H94" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I94" s="35" t="s">
+      <c r="I94" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J94" s="32"/>
-      <c r="K94" s="32"/>
-      <c r="L94" s="32"/>
-      <c r="M94" s="32"/>
-      <c r="N94" s="32"/>
-      <c r="O94" s="32"/>
-      <c r="P94" s="32"/>
-      <c r="Q94" s="32"/>
-      <c r="R94" s="32"/>
-      <c r="S94" s="32"/>
-    </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" s="9" t="s">
         <v>220</v>
       </c>
@@ -33305,21 +32536,11 @@
       <c r="H95" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I95" s="35" t="s">
+      <c r="I95" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J95" s="32"/>
-      <c r="K95" s="32"/>
-      <c r="L95" s="32"/>
-      <c r="M95" s="32"/>
-      <c r="N95" s="32"/>
-      <c r="O95" s="32"/>
-      <c r="P95" s="32"/>
-      <c r="Q95" s="32"/>
-      <c r="R95" s="32"/>
-      <c r="S95" s="32"/>
-    </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96" s="9" t="s">
         <v>222</v>
       </c>
@@ -33344,21 +32565,11 @@
       <c r="H96" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I96" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J96" s="32"/>
-      <c r="K96" s="32"/>
-      <c r="L96" s="32"/>
-      <c r="M96" s="32"/>
-      <c r="N96" s="32"/>
-      <c r="O96" s="32"/>
-      <c r="P96" s="32"/>
-      <c r="Q96" s="32"/>
-      <c r="R96" s="32"/>
-      <c r="S96" s="32"/>
-    </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I96" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" s="9" t="s">
         <v>224</v>
       </c>
@@ -33383,21 +32594,11 @@
       <c r="H97" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I97" s="35" t="s">
+      <c r="I97" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J97" s="32"/>
-      <c r="K97" s="32"/>
-      <c r="L97" s="32"/>
-      <c r="M97" s="32"/>
-      <c r="N97" s="32"/>
-      <c r="O97" s="32"/>
-      <c r="P97" s="32"/>
-      <c r="Q97" s="32"/>
-      <c r="R97" s="32"/>
-      <c r="S97" s="32"/>
-    </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" s="9" t="s">
         <v>226</v>
       </c>
@@ -33422,21 +32623,11 @@
       <c r="H98" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I98" s="35" t="s">
+      <c r="I98" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J98" s="32"/>
-      <c r="K98" s="32"/>
-      <c r="L98" s="32"/>
-      <c r="M98" s="32"/>
-      <c r="N98" s="32"/>
-      <c r="O98" s="32"/>
-      <c r="P98" s="32"/>
-      <c r="Q98" s="32"/>
-      <c r="R98" s="32"/>
-      <c r="S98" s="32"/>
-    </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" s="9" t="s">
         <v>228</v>
       </c>
@@ -33461,21 +32652,11 @@
       <c r="H99" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I99" s="35" t="s">
+      <c r="I99" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J99" s="32"/>
-      <c r="K99" s="32"/>
-      <c r="L99" s="32"/>
-      <c r="M99" s="32"/>
-      <c r="N99" s="32"/>
-      <c r="O99" s="32"/>
-      <c r="P99" s="32"/>
-      <c r="Q99" s="32"/>
-      <c r="R99" s="32"/>
-      <c r="S99" s="32"/>
-    </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" s="9" t="s">
         <v>230</v>
       </c>
@@ -33500,21 +32681,11 @@
       <c r="H100" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I100" s="35" t="s">
+      <c r="I100" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J100" s="32"/>
-      <c r="K100" s="32"/>
-      <c r="L100" s="32"/>
-      <c r="M100" s="32"/>
-      <c r="N100" s="32"/>
-      <c r="O100" s="32"/>
-      <c r="P100" s="32"/>
-      <c r="Q100" s="32"/>
-      <c r="R100" s="32"/>
-      <c r="S100" s="32"/>
-    </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" s="9" t="s">
         <v>232</v>
       </c>
@@ -33539,21 +32710,11 @@
       <c r="H101" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I101" s="35" t="s">
+      <c r="I101" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J101" s="32"/>
-      <c r="K101" s="32"/>
-      <c r="L101" s="32"/>
-      <c r="M101" s="32"/>
-      <c r="N101" s="32"/>
-      <c r="O101" s="32"/>
-      <c r="P101" s="32"/>
-      <c r="Q101" s="32"/>
-      <c r="R101" s="32"/>
-      <c r="S101" s="32"/>
-    </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102" s="9" t="s">
         <v>234</v>
       </c>
@@ -33582,7 +32743,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" s="9" t="s">
         <v>236</v>
       </c>
@@ -33611,7 +32772,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" s="9" t="s">
         <v>238</v>
       </c>
@@ -33640,7 +32801,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" s="9" t="s">
         <v>240</v>
       </c>
@@ -33669,7 +32830,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" s="9" t="s">
         <v>242</v>
       </c>
@@ -33698,7 +32859,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" s="9" t="s">
         <v>244</v>
       </c>
@@ -33727,7 +32888,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" s="9" t="s">
         <v>246</v>
       </c>
@@ -33756,7 +32917,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" s="9" t="s">
         <v>248</v>
       </c>
@@ -33785,7 +32946,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110" s="9" t="s">
         <v>250</v>
       </c>
@@ -33814,7 +32975,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" s="9" t="s">
         <v>252</v>
       </c>
@@ -33843,7 +33004,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" s="9" t="s">
         <v>254</v>
       </c>
@@ -39376,12 +38537,12 @@
       <c r="I2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="26" t="s">
         <v>634</v>
       </c>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="24"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
       <c r="O2" s="17"/>
       <c r="P2" s="17"/>
       <c r="Q2" s="17"/>
@@ -39415,10 +38576,10 @@
       <c r="I3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="27"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="31"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -39448,10 +38609,10 @@
       <c r="I4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="31"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -39481,10 +38642,10 @@
       <c r="I5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="25"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
@@ -39514,10 +38675,10 @@
       <c r="I6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="28"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="30"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="34"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
@@ -48142,11 +47303,11 @@
         <f>E2-D2</f>
         <v>1</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="26" t="s">
         <v>635</v>
       </c>
-      <c r="M2" s="23"/>
-      <c r="N2" s="24"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -48180,9 +47341,9 @@
         <f t="shared" ref="J3:J66" si="0">E3-D3</f>
         <v>7</v>
       </c>
-      <c r="L3" s="25"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="27"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="31"/>
     </row>
     <row r="4" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -48216,9 +47377,9 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="L4" s="25"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="31"/>
       <c r="O4" s="17"/>
       <c r="P4" s="17"/>
       <c r="Q4" s="17"/>
@@ -48261,9 +47422,9 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="L5" s="25"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
@@ -48297,9 +47458,9 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="L6" s="28"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="30"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="34"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
@@ -58052,7 +57213,7 @@
         <f t="shared" ref="K3:K6" si="0">F3-E3</f>
         <v>7</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="35" t="s">
         <v>642</v>
       </c>
     </row>
@@ -58156,6 +57317,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="O3" r:id="rId1" xr:uid="{B23B4049-7BF6-44C7-99BF-F514A27E6030}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -58241,12 +57405,12 @@
         <f>E2-D2</f>
         <v>1</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="26" t="s">
         <v>633</v>
       </c>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="24"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
     </row>
     <row r="3" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -58280,10 +57444,10 @@
         <f t="shared" ref="J3:J66" si="0">E3-D3</f>
         <v>7</v>
       </c>
-      <c r="L3" s="25"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="27"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="30"/>
+      <c r="O3" s="31"/>
       <c r="P3" s="17"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
@@ -58318,10 +57482,10 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="L4" s="25"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="27"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="31"/>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
@@ -58355,10 +57519,10 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="L5" s="28"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="30"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="33"/>
+      <c r="O5" s="34"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">

</xml_diff>